<commit_message>
feat: synchronize dashboard data layers
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-09-11 19:39:04 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-09-13 16:53:36 | 数据源: Shioaji Snapshot | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -738,10 +738,10 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>• 毛利率：65.0% - 67.0%
-• 净利率：&gt;43.0%
-• ROE：40.5%
-• EPS：22.08 元 (26Q1)</t>
+          <t>• 毛利率：67.03% (2026Q2)
+• 净利率：53.22% (2026Q2)
+• ROE：79.5% (單季年化, 2026Q2)
+• EPS：49.33 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -751,15 +751,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>外资: +3031 张
-投信: -1765 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+3,031 张)，投信阶段获利减仓 (-1,765 张)。</t>
+          <t>外资: -8252 张
+投信: -181 张
+[2026-09-11 官方结算] 三大法人同步卖超 (-8,833 张)，短线筹码面临清洗。</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 1,243 张 (占量 9.2%)
-[2026-08-28 筹码] 主力机构呈净买入 (+1,243 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 8,833 张 (占量 48.8%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-8,833 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -825,10 +825,10 @@
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>• 毛利率：87.0%
-• 净利率：&gt;52.0%
-• ROE：21.72%
-• EPS：74.38 元 (26Q2)</t>
+          <t>• 毛利率：84.18% (2026Q2)
+• 净利率：64.95% (2026Q2)
+• ROE：125.3% (單季年化, 2026Q2)
+• EPS：110.96 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
@@ -838,15 +838,15 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>外资: +102 张
-投信: -59 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+102 张)，投信阶段获利减仓 (-59 张)。</t>
+          <t>外资: +60 张
+投信: -36 张
+[2026-09-11 官方结算] 外资主力大幅回流 (+60 张)，投信阶段获利减仓 (-36 张)。</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 34 张 (占量 8.8%)
-[2026-08-28 筹码] 主力机构呈净买入 (+34 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净买超 16 张 (占量 4.6%)
+[2026-09-11 筹码] 主力机构呈净买入 (+16 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -912,10 +912,10 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>• 毛利率：33.8%
-• 净利率：~19.5%
-• ROE：18.58%
-• EPS：27.55 元 (26Q2)</t>
+          <t>• 毛利率：32.03% (2026Q2)
+• 净利率：18.93% (2026Q2)
+• ROE：104.3% (單季年化, 2026Q2)
+• EPS：42.46 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -925,15 +925,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>外资: +45 张
-投信: -172 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+45 张)，投信阶段获利减仓 (-172 张)。</t>
+          <t>外资: -23 张
+投信: +110 张
+[2026-09-11 官方结算] 投信内资买超 (+110 张) 逢低承接，外资高档调节 (-23 张)。</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 152 张 (占量 8.2%)
-[2026-08-28 筹码] 主力机构呈净卖出 (-152 张)，散户承接，筹码短期发散。</t>
+          <t>法人净买超 69 张 (占量 6.7%)
+[2026-09-11 筹码] 主力机构呈净买入 (+69 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -999,10 +999,10 @@
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>• 毛利率：33.8% - 35.0%
-• 净利率：~14.2%
-• ROE：17.03%
-• EPS：20.17 元 (26Q1)</t>
+          <t>• 毛利率：31.17% (2026Q2)
+• 净利率：19.31% (2026Q2)
+• ROE：126.7% (單季年化, 2026Q2)
+• EPS：44.54 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -1012,15 +1012,15 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>外资: -34 张
-投信: +626 张
-[2026-08-28 官方结算] 投信内资买超 (+626 张) 逢低承接，外资高档调节 (-34 张)。</t>
+          <t>外资: -99 张
+投信: +45 张
+[2026-09-11 官方结算] 投信内资买超 (+45 张) 逢低承接，外资高档调节 (-99 张)。</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 503 张 (占量 13.2%)
-[2026-08-28 筹码] 主力机构呈净买入 (+503 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 94 张 (占量 4.7%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-94 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1086,28 +1086,28 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>• 毛利率：6.2% - 6.8%
-• 净利率：~2.8%
-• ROE：11.25%
-• EPS：3.23 元 (25Q4)</t>
+          <t>• 毛利率：6.15% (2026Q2)
+• 净利率：2.73% (2026Q2)
+• ROE：23.0% (單季年化, 2026Q2)
+• EPS：7.84 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14 (26Q2 法说会 - 本周五) | 每月 5 日发布营收</t>
+          <t>2026-08-14 (26Q2 法說會已舉行)；下一次財報/法說會日期待公司公告 | 每月 5 日发布营收</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>外资: +1192 张
-投信: +307 张
-[2026-08-28 官方结算] 外资与投信联手买超 (+776 张)，内外部机构共振做多。</t>
+          <t>外资: -3751 张
+投信: +410 张
+[2026-09-11 官方结算] 投信内资买超 (+410 张) 逢低承接，外资高档调节 (-3,751 张)。</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 776 张 (占量 2.5%)
-[2026-08-28 筹码] 主力机构呈净买入 (+776 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 3,386 张 (占量 14.4%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-3,386 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1173,10 +1173,10 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>• 毛利率：35.6% (26Q2)
-• 净利率：13.7% (26Q2)
-• ROE：待更新
-• EPS：9.68 元 (26Q2)</t>
+          <t>• 毛利率：36.27% (2026Q2)
+• 净利率：14.89% (2026Q2)
+• ROE：62.2% (單季年化, 2026Q2)
+• EPS：17.59 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F9" s="16" t="inlineStr">
@@ -1186,15 +1186,15 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>外资: +1163 张
-投信: -732 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+1,163 张)，投信阶段获利减仓 (-732 张)。</t>
+          <t>外资: -3573 张
+投信: -536 张
+[2026-09-11 官方结算] 外资与投信偏空调节 (-3,805 张)，机构筹码阶段获利了结。</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 546 张 (占量 4.4%)
-[2026-08-28 筹码] 主力机构呈净买入 (+546 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 3,805 张 (占量 27.6%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-3,805 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
@@ -1260,10 +1260,10 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>• 毛利率：19.7% (26Q2)
-• 净利率：約 11.6% (26Q2)
-• ROE：待更新
-• EPS：19.78 元 (26Q2)</t>
+          <t>• 毛利率：19.63% (2026Q2)
+• 净利率：11.70% (2026Q2)
+• ROE：112.4% (單季年化, 2026Q2)
+• EPS：34.70 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1273,15 +1273,15 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>外资: -532 张
-投信: -18 张
-[2026-08-28 官方结算] 三大法人同步卖超 (-554 张)，短线筹码面临清洗。</t>
+          <t>外资: +572 张
+投信: -652 张
+[2026-09-11 官方结算] 外资主力大幅回流 (+572 张)，投信阶段获利减仓 (-652 张)。</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 554 张 (占量 24.7%)
-[2026-08-28 筹码] 主力机构呈净卖出 (-554 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 87 张 (占量 2.6%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-87 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1347,10 +1347,10 @@
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>• 毛利率：約 60.5% (26Q2)
-• 净利率：約 37.9% (26Q2)
-• ROE：待更新
-• EPS：約 12.15 元 (26Q2)</t>
+          <t>• 毛利率：61.48% (2026Q2)
+• 净利率：36.15% (2026Q2)
+• ROE：109.0% (單季年化, 2026Q2)
+• EPS：21.27 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
@@ -1360,15 +1360,15 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>外资: +57 张
-投信: -33 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+57 张)，投信阶段获利减仓 (-33 张)。</t>
+          <t>外资: +143 张
+投信: +92 张
+[2026-09-11 官方结算] 外资与投信联手买超 (+225 张)，内外部机构共振做多。</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 12 张 (占量 0.8%)
-[2026-08-28 筹码] 主力机构呈净买入 (+12 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净买超 225 张 (占量 10.2%)
+[2026-09-11 筹码] 主力机构呈净买入 (+225 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -1434,10 +1434,10 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>• 毛利率：待更新
-• 净利率：約 11.0% (26Q2)
-• ROE：18.2% 年化 (26H1)
-• EPS：4.80 元 (26Q2)</t>
+          <t>• 毛利率：20.55% (2026Q2)
+• 净利率：9.89% (2026Q2)
+• ROE：36.2% (單季年化, 2026Q2)
+• EPS：8.04 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1447,15 +1447,15 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>外资: -568 张
-投信: +61 张
-[2026-08-28 官方结算] 投信内资买超 (+61 张) 逢低承接，外资高档调节 (-568 张)。</t>
+          <t>外资: -8053 张
+投信: +679 张
+[2026-09-11 官方结算] 投信内资买超 (+679 张) 逢低承接，外资高档调节 (-8,053 张)。</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 440 张 (占量 2.5%)
-[2026-08-28 筹码] 主力机构呈净买入 (+440 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 7,819 张 (占量 36.3%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-7,819 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1521,10 +1521,10 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>• 毛利率：46.2% (26Q2)
-• 净利率：約 16.2% (26Q2)
-• ROE：待更新
-• EPS：15.28 元 (26Q2)</t>
+          <t>• 毛利率：46.25% (2026Q2)
+• 净利率：16.25% (2026Q2)
+• ROE：45.7% (單季年化, 2026Q2)
+• EPS：30.44 元 (2026Q2)</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -1534,15 +1534,15 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>外资: +1096 张
-投信: -118 张
-[2026-08-28 官方结算] 外资主力大幅回流 (+1,096 张)，投信阶段获利减仓 (-118 张)。</t>
+          <t>外资: -743 张
+投信: +108 张
+[2026-09-11 官方结算] 投信内资买超 (+108 张) 逢低承接，外资高档调节 (-743 张)。</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 996 张 (占量 23.8%)
-[2026-08-28 筹码] 主力机构呈净买入 (+996 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 656 张 (占量 9.6%)
+[2026-09-11 筹码] 主力机构呈净卖出 (-656 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-11 19:39:04 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-13 16:53:36 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish verified September 16 close
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-09-16 19:53:41 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-09-16 20:18:39 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-16 19:53:41 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-16 20:18:39 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: refresh complete official institutional flows
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-09-16 20:18:39 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-09-16 20:27:43 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -751,15 +751,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>外资: -8252 张
-投信: -181 张
-[2026-09-11 官方结算] 三大法人同步卖超 (-8,833 张)，短线筹码面临清洗。</t>
+          <t>外资: -8745 张
+投信: +166 张
+[2026-09-16 官方结算] 投信内资买超 (+166 张) 逢低承接，外资高档调节 (-8,745 张)。</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 8,833 张 (占量 48.8%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-8,833 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 7,816 张 (占量 43.5%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-7,816 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -838,15 +838,15 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>外资: +60 张
-投信: -36 张
-[2026-09-11 官方结算] 外资主力大幅回流 (+60 张)，投信阶段获利减仓 (-36 张)。</t>
+          <t>外资: -64 张
+投信: +59 张
+[2026-09-16 官方结算] 投信内资买超 (+59 张) 逢低承接，外资高档调节 (-64 张)。</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 16 张 (占量 4.6%)
-[2026-09-11 筹码] 主力机构呈净买入 (+16 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 30 张 (占量 7.2%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-30 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -925,15 +925,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>外资: -23 张
-投信: +110 张
-[2026-09-11 官方结算] 投信内资买超 (+110 张) 逢低承接，外资高档调节 (-23 张)。</t>
+          <t>外资: +67 张
+投信: -147 张
+[2026-09-16 官方结算] 外资主力大幅回流 (+67 张)，投信阶段获利减仓 (-147 张)。</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 69 张 (占量 6.7%)
-[2026-09-11 筹码] 主力机构呈净买入 (+69 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 154 张 (占量 10.1%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-154 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -1012,15 +1012,15 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>外资: -99 张
-投信: +45 张
-[2026-09-11 官方结算] 投信内资买超 (+45 张) 逢低承接，外资高档调节 (-99 张)。</t>
+          <t>外资: -201 张
+投信: +80 张
+[2026-09-16 官方结算] 投信内资买超 (+80 张) 逢低承接，外资高档调节 (-201 张)。</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 94 张 (占量 4.7%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-94 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 91 张 (占量 3.5%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-91 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1099,15 +1099,15 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>外资: -3751 张
-投信: +410 张
-[2026-09-11 官方结算] 投信内资买超 (+410 张) 逢低承接，外资高档调节 (-3,751 张)。</t>
+          <t>外资: -1689 张
+投信: +1281 张
+[2026-09-16 官方结算] 投信内资买超 (+1,281 张) 逢低承接，外资高档调节 (-1,689 张)。</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 3,386 张 (占量 14.4%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-3,386 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 2,590 张 (占量 13.4%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-2,590 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1186,15 +1186,15 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>外资: -3573 张
-投信: -536 张
-[2026-09-11 官方结算] 外资与投信偏空调节 (-3,805 张)，机构筹码阶段获利了结。</t>
+          <t>外资: -845 张
+投信: +551 张
+[2026-09-16 官方结算] 投信内资买超 (+551 张) 逢低承接，外资高档调节 (-845 张)。</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 3,805 张 (占量 27.6%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-3,805 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 567 张 (占量 5.7%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-567 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
@@ -1273,15 +1273,15 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>外资: +572 张
-投信: -652 张
-[2026-09-11 官方结算] 外资主力大幅回流 (+572 张)，投信阶段获利减仓 (-652 张)。</t>
+          <t>外资: -259 张
+投信: -129 张
+[2026-09-16 官方结算] 三大法人同步卖超 (-500 张)，短线筹码面临清洗。</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 87 张 (占量 2.6%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-87 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 500 张 (占量 21.6%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-500 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1360,15 +1360,15 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>外资: +143 张
-投信: +92 张
-[2026-09-11 官方结算] 外资与投信联手买超 (+225 张)，内外部机构共振做多。</t>
+          <t>外资: -104 张
+投信: +25 张
+[2026-09-16 官方结算] 投信内资买超 (+25 张) 逢低承接，外资高档调节 (-104 张)。</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 225 张 (占量 10.2%)
-[2026-09-11 筹码] 主力机构呈净买入 (+225 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 76 张 (占量 7.1%)
+[2026-09-16 筹码] 主力机构呈净卖出 (-76 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -1447,15 +1447,15 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>外资: -8053 张
-投信: +679 张
-[2026-09-11 官方结算] 投信内资买超 (+679 张) 逢低承接，外资高档调节 (-8,053 张)。</t>
+          <t>外资: +2606 张
+投信: -1038 张
+[2026-09-16 官方结算] 外资主力大幅回流 (+2,606 张)，投信阶段获利减仓 (-1,038 张)。</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 7,819 张 (占量 36.3%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-7,819 张)，散户承接，筹码短期发散。</t>
+          <t>法人净买超 1,663 张 (占量 18.5%)
+[2026-09-16 筹码] 主力机构呈净买入 (+1,663 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1534,15 +1534,15 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>外资: -743 张
-投信: +108 张
-[2026-09-11 官方结算] 投信内资买超 (+108 张) 逢低承接，外资高档调节 (-743 张)。</t>
+          <t>外资: +997 张
+投信: -484 张
+[2026-09-16 官方结算] 外资主力大幅回流 (+997 张)，投信阶段获利减仓 (-484 张)。</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 656 张 (占量 9.6%)
-[2026-09-11 筹码] 主力机构呈净卖出 (-656 张)，散户承接，筹码短期发散。</t>
+          <t>法人净买超 729 张 (占量 12.4%)
+[2026-09-16 筹码] 主力机构呈净买入 (+729 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-16 20:18:39 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-16 20:27:43 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 11-stock dashboard snapshot
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -624,14 +624,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>台股 10 檔 AI 核心卡位龙头深度投资与买卖点筹码量化分析表</t>
+          <t>台股 11 檔 AI 核心卡位龙头深度投资与买卖点筹码量化分析表</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-09-22 19:55:29 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-09-23 14:11:55 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2505.0
-最高: 2510.0
-最低: 2460.0
-收盘: 2460.0</t>
+          <t>开盘: 2475.0
+最高: 2505.0
+最低: 2475.0
+收盘: 2500.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 4,268 张 (占量 22.6%)
+          <t>法人净卖超 4,268 张 (占量 21.0%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-4,268 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2460.0</t>
+          <t>NT$ 2500.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>18,900 张</t>
+          <t>20,325 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 12900.0
-最高: 13305.0
-最低: 12670.0
-收盘: 12670.0</t>
+          <t>开盘: 12670.0
+最高: 12725.0
+最低: 12320.0
+收盘: 12390.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 42 张 (占量 10.9%)
+          <t>法人净卖超 42 张 (占量 13.6%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-42 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 12670.0</t>
+          <t>NT$ 12390.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>384 张</t>
+          <t>309 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5100.0
-最高: 5100.0
-最低: 4855.0
-收盘: 4860.0</t>
+          <t>开盘: 4910.0
+最高: 5110.0
+最低: 4860.0
+收盘: 5020.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 273 张 (占量 16.2%)
+          <t>法人净卖超 273 张 (占量 12.2%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-273 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4860.0</t>
+          <t>NT$ 5020.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>1,685 张</t>
+          <t>2,241 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3500.0
-最高: 3505.0
-最低: 3385.0
-收盘: 3390.0</t>
+          <t>开盘: 3425.0
+最高: 3590.0
+最低: 3410.0
+收盘: 3470.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 195 张 (占量 9.0%)
+          <t>法人净卖超 195 张 (占量 7.8%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-195 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3390.0</t>
+          <t>NT$ 3470.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,168 张</t>
+          <t>2,485 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 252.0
-最高: 254.0
-最低: 250.5
-收盘: 253.0</t>
+          <t>开盘: 255.0
+最高: 257.0
+最低: 255.0
+收盘: 256.0</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 7,725 张 (占量 20.5%)
+          <t>法人净买超 7,725 张 (占量 22.3%)
 [2026-09-22 筹码] 主力机构呈净买入 (+7,725 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 253.0</t>
+          <t>NT$ 256.0</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>37,621 张</t>
+          <t>34,627 张</t>
         </is>
       </c>
     </row>
@@ -1165,9 +1165,9 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1965.0
-最高: 1965.0
-最低: 1900.0
+          <t>开盘: 1910.0
+最高: 1920.0
+最低: 1890.0
 收盘: 1900.0</t>
         </is>
       </c>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 311 张 (占量 2.0%)
+          <t>法人净买超 311 张 (占量 3.5%)
 [2026-09-22 筹码] 主力机构呈净买入 (+311 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>15,381 张</t>
+          <t>9,000 张</t>
         </is>
       </c>
     </row>
@@ -1252,10 +1252,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 1900.0
-最高: 1935.0
-最低: 1865.0
-收盘: 1915.0</t>
+          <t>开盘: 1935.0
+最高: 1955.0
+最低: 1845.0
+收盘: 1890.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 272 张 (占量 7.3%)
+          <t>法人净卖超 272 张 (占量 7.0%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-272 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1915.0</t>
+          <t>NT$ 1890.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>3,714 张</t>
+          <t>3,860 张</t>
         </is>
       </c>
     </row>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>开盘: 2395.0
-最高: 2540.0
-最低: 2350.0
-收盘: 2440.0</t>
+          <t>开盘: 2445.0
+最高: 2470.0
+最低: 2305.0
+收盘: 2325.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 72 张 (占量 2.6%)
+          <t>法人净卖超 72 张 (占量 2.9%)
 [2026-09-22 筹码] 主力机构呈净卖出 (-72 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2440.0</t>
+          <t>NT$ 2325.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>2,759 张</t>
+          <t>2,511 张</t>
         </is>
       </c>
     </row>
@@ -1426,9 +1426,9 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 691.0
+          <t>开盘: 710.0
 最高: 711.0
-最低: 690.0
+最低: 689.0
 收盘: 693.0</t>
         </is>
       </c>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 10,751 张 (占量 47.9%)
+          <t>法人净买超 10,751 张 (占量 73.8%)
 [2026-09-22 筹码] 主力机构呈净买入 (+10,751 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>22,466 张</t>
+          <t>14,576 张</t>
         </is>
       </c>
     </row>
@@ -1513,10 +1513,10 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 5280.0
-最高: 5480.0
-最低: 5150.0
-收盘: 5180.0</t>
+          <t>开盘: 5220.0
+最高: 5265.0
+最低: 5140.0
+收盘: 5185.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 1,972 张 (占量 18.7%)
+          <t>法人净买超 1,972 张 (占量 33.4%)
 [2026-09-22 筹码] 主力机构呈净买入 (+1,972 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 5180.0</t>
+          <t>NT$ 5185.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,94 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>10,528 张</t>
+          <t>5,902 张</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3653.TW</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>健策</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>由封裝端均熱片、VC／微流道蓋板到系統端液冷冷板的垂直熱管理產品鏈</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>开盘: 6005.0
+最高: 6410.0
+最低: 5930.0
+收盘: 6410.0</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>• 毛利率：46.81% (2026Q2)
+• 净利率：32.01% (2026Q2)
+• ROE：63.1% (單季年化, 2026Q2)
+• EPS：15.80 元 (2026Q2)</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>2026Q2 已公告；下一次財報/法說日待公司公告</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>外资: -201 张
+投信: +85 张
+[2026-09-22 官方结算] 投信内资买超 (+85 张) 逢低承接，外资高档调节 (-201 张)。</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>法人净卖超 119 张 (占量 8.5%)
+[2026-09-22 筹码] 主力机构呈净卖出 (-119 张)，散户承接，筹码短期发散。</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>【Chokepoint 88分】卡位最上游铲子卖家，客户切换周期超 12-36 个月，垄断护城河极深。</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 6410.0</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>建议买点：待估值與技術面複核
+黄金重仓：暫不設定</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>依獲利與估值重新評估</t>
+        </is>
+      </c>
+      <c r="M14" s="11" t="inlineStr">
+        <is>
+          <t>不預設固定目標</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr">
+        <is>
+          <t>依獲利趨勢與個人風險承受度管理</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>1,394 张</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1614,14 +1701,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>台股 10 檔卡位龙头 Shioaji 实时买卖点与风控决策面板</t>
+          <t>台股 11 檔卡位龙头 Shioaji 实时买卖点与风控决策面板</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-22 19:55:29 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-09-23 14:11:55 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1685,22 +1772,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
+          <t>NT$ 2475.0</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
           <t>NT$ 2505.0</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2510.0</t>
-        </is>
-      </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2460.0</t>
+          <t>NT$ 2475.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2460.0</t>
+          <t>NT$ 2500.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1732,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 12900.0</t>
+          <t>NT$ 12670.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 13305.0</t>
+          <t>NT$ 12725.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 12670.0</t>
+          <t>NT$ 12320.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 12670.0</t>
+          <t>NT$ 12390.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1779,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5100.0</t>
+          <t>NT$ 4910.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5100.0</t>
+          <t>NT$ 5110.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 4855.0</t>
+          <t>NT$ 4860.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4860.0</t>
+          <t>NT$ 5020.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1826,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3500.0</t>
+          <t>NT$ 3425.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3505.0</t>
+          <t>NT$ 3590.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3385.0</t>
+          <t>NT$ 3410.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3390.0</t>
+          <t>NT$ 3470.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1873,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 252.0</t>
+          <t>NT$ 255.0</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 254.0</t>
+          <t>NT$ 257.0</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 250.5</t>
+          <t>NT$ 255.0</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 253.0</t>
+          <t>NT$ 256.0</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -1920,17 +2007,17 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1965.0</t>
+          <t>NT$ 1910.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1965.0</t>
+          <t>NT$ 1920.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1900.0</t>
+          <t>NT$ 1890.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
@@ -1967,22 +2054,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1900.0</t>
+          <t>NT$ 1935.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1935.0</t>
+          <t>NT$ 1955.0</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1865.0</t>
+          <t>NT$ 1845.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1915.0</t>
+          <t>NT$ 1890.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2014,22 +2101,22 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2395.0</t>
+          <t>NT$ 2445.0</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2540.0</t>
+          <t>NT$ 2470.0</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2350.0</t>
+          <t>NT$ 2305.0</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2440.0</t>
+          <t>NT$ 2325.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2061,7 +2148,7 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 691.0</t>
+          <t>NT$ 710.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
@@ -2071,7 +2158,7 @@
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 690.0</t>
+          <t>NT$ 689.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -2108,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 5280.0</t>
+          <t>NT$ 5220.0</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 5480.0</t>
+          <t>NT$ 5265.0</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 5150.0</t>
+          <t>NT$ 5140.0</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 5180.0</t>
+          <t>NT$ 5185.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2139,6 +2226,53 @@
       <c r="I13" s="17" t="inlineStr">
         <is>
           <t>獲利與 ASIC 時程轉弱即檢視</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>3653.TW</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>健策</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 6005.0</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 6410.0</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 5930.0</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>NT$ 6410.0</t>
+        </is>
+      </c>
+      <c r="G14" s="25" t="inlineStr">
+        <is>
+          <t>待估值與技術面複核</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>依獲利與估值重新評估</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>依獲利趨勢與個人風險承受度管理</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: publish refreshed stock content and freshness metadata
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-16 19:43:44 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-19 20:33:54 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,9 +730,9 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2430.0
-最高: 2445.0
-最低: 2420.0
+          <t>开盘: 2395.0
+最高: 2420.0
+最低: 2390.0
 收盘: 2420.0</t>
         </is>
       </c>
@@ -740,7 +740,7 @@
         <is>
           <t>• 毛利率：67.03% (2026Q2)
 • 净利率：53.22% (2026Q2)
-• ROE：79.5% (單季年化, 2026Q2)
+• ROE：39.8% (年初累計年化, 2026Q2)
 • EPS：27.25 元 (2026Q2 單季；TSMC 官方財報)</t>
         </is>
       </c>
@@ -751,15 +751,15 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>外资: -22047 张
-投信: +710 张
-[2026-10-16 官方结算] 投信内资买超 (+710 张) 逢低承接，外资高档调节 (-22,047 张)。</t>
+          <t>外资: -9835 张
+投信: +3884 张
+[2026-10-19 官方结算] 投信内资买超 (+3,884 张) 逢低承接，外资高档调节 (-9,835 张)。</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 22,372 张 (占量 67.0%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-22,372 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 4,604 张 (占量 19.5%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-4,604 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>33,389 张</t>
+          <t>23,643 张</t>
         </is>
       </c>
     </row>
@@ -817,17 +817,17 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 10140.0
-最高: 10175.0
-最低: 9775.0
-收盘: 9955.0</t>
+          <t>开盘: 9785.0
+最高: 10040.0
+最低: 9690.0
+收盘: 9920.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
           <t>• 毛利率：84.18% (2026Q2)
 • 净利率：64.95% (2026Q2)
-• ROE：125.3% (單季年化, 2026Q2)
+• ROE：62.7% (年初累計年化, 2026Q2)
 • EPS：74.38 元 (2026Q2 單季；公司法說資料)</t>
         </is>
       </c>
@@ -838,15 +838,15 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>外资: -141 张
-投信: +47 张
-[2026-10-16 官方结算] 投信内资买超 (+47 张) 逢低承接，外资高档调节 (-141 张)。</t>
+          <t>外资: -60 张
+投信: +9 张
+[2026-10-19 官方结算] 投信内资买超 (+9 张) 逢低承接，外资高档调节 (-60 张)。</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 109 张 (占量 20.8%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-109 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 52 张 (占量 13.9%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-52 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I5" s="15" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9955.0</t>
+          <t>NT$ 9920.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>523 张</t>
+          <t>373 张</t>
         </is>
       </c>
     </row>
@@ -904,17 +904,17 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5155.0
-最高: 5260.0
-最低: 5005.0
-收盘: 5165.0</t>
+          <t>开盘: 5010.0
+最高: 5165.0
+最低: 4955.0
+收盘: 5125.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
           <t>• 毛利率：32.03% (2026Q2)
 • 净利率：18.93% (2026Q2)
-• ROE：104.3% (單季年化, 2026Q2)
+• ROE：52.2% (年初累計年化, 2026Q2)
 • EPS：27.55 元 (2026Q2 單季；公司季度財報)</t>
         </is>
       </c>
@@ -925,15 +925,15 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>外资: +196 张
-投信: -186 张
-[2026-10-16 官方结算] 外资主力大幅回流 (+196 张)，投信阶段获利减仓 (-186 张)。</t>
+          <t>外资: +16 张
+投信: +15 张
+[2026-10-19 官方结算] 外资与投信联手买超 (+-80 张)，内外部机构共振做多。</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 63 张 (占量 2.5%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-63 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 80 张 (占量 5.0%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-80 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5165.0</t>
+          <t>NT$ 5125.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>2,552 张</t>
+          <t>1,604 张</t>
         </is>
       </c>
     </row>
@@ -991,17 +991,17 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3115.0
-最高: 3355.0
-最低: 3080.0
-收盘: 3315.0</t>
+          <t>开盘: 3220.0
+最高: 3350.0
+最低: 3180.0
+收盘: 3320.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
           <t>• 毛利率：31.17% (2026Q2)
 • 净利率：19.31% (2026Q2)
-• ROE：126.7% (單季年化, 2026Q2)
+• ROE：63.3% (年初累計年化, 2026Q2)
 • EPS：24.37 元 (2026Q2 單季；公司季度財報)</t>
         </is>
       </c>
@@ -1012,15 +1012,15 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>外资: -725 张
-投信: +591 张
-[2026-10-16 官方结算] 投信内资买超 (+591 张) 逢低承接，外资高档调节 (-725 张)。</t>
+          <t>外资: -527 张
+投信: +509 张
+[2026-10-19 官方结算] 投信内资买超 (+509 张) 逢低承接，外资高档调节 (-527 张)。</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 154 张 (占量 4.3%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-154 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 24 张 (占量 1.0%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-24 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I7" s="15" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3315.0</t>
+          <t>NT$ 3320.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>3,568 张</t>
+          <t>2,319 张</t>
         </is>
       </c>
     </row>
@@ -1078,17 +1078,17 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 241.5
-最高: 247.0
-最低: 240.5
-收盘: 244.0</t>
+          <t>开盘: 242.0
+最高: 242.5
+最低: 238.5
+收盘: 239.5</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>• 毛利率：6.15% (2026Q2)
 • 净利率：2.73% (2026Q2)
-• ROE：23.0% (單季年化, 2026Q2)
+• ROE：11.5% (年初累計年化, 2026Q2)
 • EPS：4.27 元 (2026Q2 單季；鴻海官方公告)</t>
         </is>
       </c>
@@ -1099,15 +1099,15 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>外资: +22670 张
-投信: -239 张
-[2026-10-16 官方结算] 外资主力大幅回流 (+22,670 张)，投信阶段获利减仓 (-239 张)。</t>
+          <t>外资: -14885 张
+投信: +817 张
+[2026-10-19 官方结算] 投信内资买超 (+817 张) 逢低承接，外资高档调节 (-14,885 张)。</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 23,159 张 (占量 47.0%)
-[2026-10-16 筹码] 主力机构呈净买入 (+23,159 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净卖超 13,522 张 (占量 46.2%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-13,522 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 244.0</t>
+          <t>NT$ 239.5</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>49,268 张</t>
+          <t>29,293 张</t>
         </is>
       </c>
     </row>
@@ -1165,17 +1165,17 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1650.0
-最高: 1665.0
-最低: 1630.0
-收盘: 1635.0</t>
+          <t>开盘: 1600.0
+最高: 1655.0
+最低: 1590.0
+收盘: 1640.0</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
           <t>• 毛利率：36.27% (2026Q2)
 • 净利率：14.89% (2026Q2)
-• ROE：62.2% (單季年化, 2026Q2)
+• ROE：31.1% (年初累計年化, 2026Q2)
 • EPS：9.68 元 (26Q2)</t>
         </is>
       </c>
@@ -1186,15 +1186,15 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>外资: -2134 张
-投信: +268 张
-[2026-10-16 官方结算] 投信内资买超 (+268 张) 逢低承接，外资高档调节 (-2,134 张)。</t>
+          <t>外资: -835 张
+投信: +632 张
+[2026-10-19 官方结算] 投信内资买超 (+632 张) 逢低承接，外资高档调节 (-835 张)。</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 2,005 张 (占量 27.1%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-2,005 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 782 张 (占量 11.2%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-782 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I9" s="15" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1635.0</t>
+          <t>NT$ 1640.0</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>7,388 张</t>
+          <t>6,954 张</t>
         </is>
       </c>
     </row>
@@ -1252,17 +1252,17 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 1965.0
-最高: 2030.0
-最低: 1935.0
-收盘: 1980.0</t>
+          <t>开盘: 1925.0
+最高: 2055.0
+最低: 1910.0
+收盘: 2005.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>• 毛利率：19.63% (2026Q2)
 • 净利率：11.70% (2026Q2)
-• ROE：112.4% (單季年化, 2026Q2)
+• ROE：56.2% (年初累計年化, 2026Q2)
 • EPS：19.78 元 (26Q2)</t>
         </is>
       </c>
@@ -1273,15 +1273,15 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>外资: -63 张
-投信: +354 张
-[2026-10-16 官方结算] 投信内资买超 (+354 张) 逢低承接，外资高档调节 (-63 张)。</t>
+          <t>外资: +1008 张
+投信: -62 张
+[2026-10-19 官方结算] 外资主力大幅回流 (+1,008 张)，投信阶段获利减仓 (-62 张)。</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 305 张 (占量 9.0%)
-[2026-10-16 筹码] 主力机构呈净买入 (+305 张)，筹码向法人端汇聚沉淀。</t>
+          <t>法人净买超 918 张 (占量 20.1%)
+[2026-10-19 筹码] 主力机构呈净买入 (+918 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1980.0</t>
+          <t>NT$ 2005.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>3,397 张</t>
+          <t>4,576 张</t>
         </is>
       </c>
     </row>
@@ -1341,15 +1341,15 @@
         <is>
           <t>开盘: 1985.0
 最高: 2045.0
-最低: 1960.0
-收盘: 2000.0</t>
+最低: 1945.0
+收盘: 2005.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
           <t>• 毛利率：61.48% (2026Q2)
 • 净利率：36.15% (2026Q2)
-• ROE：109.0% (單季年化, 2026Q2)
+• ROE：54.5% (年初累計年化, 2026Q2)
 • EPS：約 12.15 元 (26Q2)</t>
         </is>
       </c>
@@ -1360,15 +1360,15 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>外资: -717 张
-投信: +134 张
-[2026-10-16 官方结算] 投信内资买超 (+134 张) 逢低承接，外资高档调节 (-717 张)。</t>
+          <t>外资: -292 张
+投信: +3 张
+[2026-10-19 官方结算] 投信内资买超 (+3 张) 逢低承接，外资高档调节 (-292 张)。</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 534 张 (占量 15.5%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-534 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 282 张 (占量 14.4%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-282 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I11" s="15" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2005.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>3,436 张</t>
+          <t>1,953 张</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1426,17 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 652.0
-最高: 678.0
-最低: 652.0
-收盘: 671.0</t>
+          <t>开盘: 640.0
+最高: 675.0
+最低: 639.0
+收盘: 670.0</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
           <t>• 毛利率：20.55% (2026Q2)
 • 净利率：9.89% (2026Q2)
-• ROE：36.2% (單季年化, 2026Q2)
+• ROE：18.1% (年初累計年化, 2026Q2)
 • EPS：4.80 元 (26Q2)</t>
         </is>
       </c>
@@ -1447,15 +1447,15 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>外资: -1531 张
-投信: -1815 张
-[2026-10-16 官方结算] 外资与投信偏空调节 (-3,188 张)，机构筹码阶段获利了结。</t>
+          <t>外资: -1627 张
+投信: +1595 张
+[2026-10-19 官方结算] 投信内资买超 (+1,595 张) 逢低承接，外资高档调节 (-1,627 张)。</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 3,188 张 (占量 17.4%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-3,188 张)，散户承接，筹码短期发散。</t>
+          <t>法人净买超 157 张 (占量 1.1%)
+[2026-10-19 筹码] 主力机构呈净买入 (+157 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 671.0</t>
+          <t>NT$ 670.0</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>18,308 张</t>
+          <t>13,999 张</t>
         </is>
       </c>
     </row>
@@ -1513,17 +1513,17 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 4275.0
-最高: 4360.0
-最低: 4240.0
-收盘: 4250.0</t>
+          <t>开盘: 4150.0
+最高: 4250.0
+最低: 4145.0
+收盘: 4205.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
           <t>• 毛利率：46.25% (2026Q2)
 • 净利率：16.25% (2026Q2)
-• ROE：45.7% (單季年化, 2026Q2)
+• ROE：22.9% (年初累計年化, 2026Q2)
 • EPS：15.28 元 (26Q2)</t>
         </is>
       </c>
@@ -1534,15 +1534,15 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>外资: -1623 张
-投信: +471 张
-[2026-10-16 官方结算] 投信内资买超 (+471 张) 逢低承接，外资高档调节 (-1,623 张)。</t>
+          <t>外资: -1154 张
+投信: +165 张
+[2026-10-19 官方结算] 投信内资买超 (+165 张) 逢低承接，外资高档调节 (-1,154 张)。</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 1,384 张 (占量 17.9%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-1,384 张)，散户承接，筹码短期发散。</t>
+          <t>法人净卖超 1,202 张 (占量 22.5%)
+[2026-10-19 筹码] 主力机构呈净卖出 (-1,202 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
       <c r="I13" s="15" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4250.0</t>
+          <t>NT$ 4205.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>7,748 张</t>
+          <t>5,350 张</t>
         </is>
       </c>
     </row>
@@ -1600,10 +1600,10 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>开盘: 6765.0
-最高: 6950.0
-最低: 6675.0
-收盘: 6730.0</t>
+          <t>开盘: 6475.0
+最高: 6590.0
+最低: 6330.0
+收盘: 6560.0</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1621,15 +1621,15 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>外资: -110 张
-投信: +50 张
-[2026-10-16 官方结算] 投信内资买超 (+50 张) 逢低承接，外资高档调节 (-110 张)。</t>
+          <t>外资: -79 张
+投信: +89 张
+[2026-10-19 官方结算] 投信内资买超 (+89 张) 逢低承接，外资高档调节 (-79 张)。</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 93 张 (占量 8.5%)
-[2026-10-16 筹码] 主力机构呈净卖出 (-93 张)，散户承接，筹码短期发散。</t>
+          <t>法人净买超 15 张 (占量 0.8%)
+[2026-10-19 筹码] 主力机构呈净买入 (+15 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6730.0</t>
+          <t>NT$ 6560.0</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>1,099 张</t>
+          <t>1,857 张</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-16 19:43:44 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-19 20:33:54 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1772,17 +1772,17 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2430.0</t>
+          <t>NT$ 2395.0</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2445.0</t>
+          <t>NT$ 2420.0</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2420.0</t>
+          <t>NT$ 2390.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 10140.0</t>
+          <t>NT$ 9785.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 10175.0</t>
+          <t>NT$ 10040.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9775.0</t>
+          <t>NT$ 9690.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9955.0</t>
+          <t>NT$ 9920.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5155.0</t>
+          <t>NT$ 5010.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5260.0</t>
+          <t>NT$ 5165.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5005.0</t>
+          <t>NT$ 4955.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5165.0</t>
+          <t>NT$ 5125.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3115.0</t>
+          <t>NT$ 3220.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3355.0</t>
+          <t>NT$ 3350.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3080.0</t>
+          <t>NT$ 3180.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3315.0</t>
+          <t>NT$ 3320.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1960,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 241.5</t>
+          <t>NT$ 242.0</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 247.0</t>
+          <t>NT$ 242.5</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 240.5</t>
+          <t>NT$ 238.5</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 244.0</t>
+          <t>NT$ 239.5</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1650.0</t>
+          <t>NT$ 1600.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1665.0</t>
+          <t>NT$ 1655.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1630.0</t>
+          <t>NT$ 1590.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1635.0</t>
+          <t>NT$ 1640.0</t>
         </is>
       </c>
       <c r="G9" s="29" t="inlineStr">
@@ -2054,22 +2054,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1965.0</t>
+          <t>NT$ 1925.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2030.0</t>
+          <t>NT$ 2055.0</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1935.0</t>
+          <t>NT$ 1910.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1980.0</t>
+          <t>NT$ 2005.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2111,12 +2111,12 @@
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1960.0</t>
+          <t>NT$ 1945.0</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2005.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 652.0</t>
+          <t>NT$ 640.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 678.0</t>
+          <t>NT$ 675.0</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 652.0</t>
+          <t>NT$ 639.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 671.0</t>
+          <t>NT$ 670.0</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4275.0</t>
+          <t>NT$ 4150.0</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4360.0</t>
+          <t>NT$ 4250.0</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4240.0</t>
+          <t>NT$ 4145.0</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4250.0</t>
+          <t>NT$ 4205.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2242,22 +2242,22 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6765.0</t>
+          <t>NT$ 6475.0</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6950.0</t>
+          <t>NT$ 6590.0</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6675.0</t>
+          <t>NT$ 6330.0</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6730.0</t>
+          <t>NT$ 6560.0</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">

</xml_diff>

<commit_message>
fix: keep daily content sync running after quote failures
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-19 20:33:54 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-19 20:41:37 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-19 20:33:54 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-19 20:41:37 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish October 20 close report with source freshness checks
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-19 21:46:09 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-20 15:06:07 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2395.0
-最高: 2420.0
-最低: 2390.0
-收盘: 2420.0</t>
+          <t>开盘: 2400.0
+最高: 2415.0
+最低: 2395.0
+收盘: 2405.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 4,604 张 (占量 19.5%)
+          <t>法人净卖超 4,604 张 (占量 27.0%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-4,604 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2420.0</t>
+          <t>NT$ 2405.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>23,643 张</t>
+          <t>17,029 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 9785.0
-最高: 10040.0
-最低: 9690.0
-收盘: 9920.0</t>
+          <t>开盘: 9985.0
+最高: 10330.0
+最低: 9970.0
+收盘: 10100.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 52 张 (占量 13.9%)
+          <t>法人净卖超 52 张 (占量 9.8%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-52 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9920.0</t>
+          <t>NT$ 10100.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>373 张</t>
+          <t>533 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5010.0
-最高: 5165.0
-最低: 4955.0
-收盘: 5125.0</t>
+          <t>开盘: 5050.0
+最高: 5200.0
+最低: 4930.0
+收盘: 4945.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5125.0</t>
+          <t>NT$ 4945.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>1,604 张</t>
+          <t>1,585 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3220.0
-最高: 3350.0
-最低: 3180.0
-收盘: 3320.0</t>
+          <t>开盘: 3290.0
+最高: 3420.0
+最低: 3270.0
+收盘: 3325.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 24 张 (占量 1.0%)
+          <t>法人净卖超 24 张 (占量 0.9%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-24 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3320.0</t>
+          <t>NT$ 3325.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,319 张</t>
+          <t>2,637 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 242.0
-最高: 242.5
-最低: 238.5
-收盘: 239.5</t>
+          <t>开盘: 238.0
+最高: 244.5
+最低: 237.0
+收盘: 241.5</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 13,522 张 (占量 46.2%)
+          <t>法人净卖超 13,522 张 (占量 51.6%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-13,522 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 239.5</t>
+          <t>NT$ 241.5</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>29,293 张</t>
+          <t>26,229 张</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1165,10 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1600.0
-最高: 1655.0
-最低: 1590.0
-收盘: 1640.0</t>
+          <t>开盘: 1635.0
+最高: 1645.0
+最低: 1595.0
+收盘: 1605.0</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 782 张 (占量 11.2%)
+          <t>法人净卖超 782 张 (占量 9.8%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-782 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1640.0</t>
+          <t>NT$ 1605.0</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>6,954 张</t>
+          <t>7,947 张</t>
         </is>
       </c>
     </row>
@@ -1252,10 +1252,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 1925.0
+          <t>开盘: 2000.0
 最高: 2055.0
-最低: 1910.0
-收盘: 2005.0</t>
+最低: 1950.0
+收盘: 1970.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 918 张 (占量 20.1%)
+          <t>法人净买超 918 张 (占量 24.3%)
 [2026-10-19 筹码] 主力机构呈净买入 (+918 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2005.0</t>
+          <t>NT$ 1970.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>4,576 张</t>
+          <t>3,781 张</t>
         </is>
       </c>
     </row>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1985.0
-最高: 2045.0
-最低: 1945.0
-收盘: 2005.0</t>
+          <t>开盘: 2000.0
+最高: 2075.0
+最低: 1990.0
+收盘: 2000.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 282 张 (占量 14.4%)
+          <t>法人净卖超 282 张 (占量 16.3%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-282 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2005.0</t>
+          <t>NT$ 2000.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>1,953 张</t>
+          <t>1,731 张</t>
         </is>
       </c>
     </row>
@@ -1426,10 +1426,10 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 640.0
-最高: 675.0
-最低: 639.0
-收盘: 670.0</t>
+          <t>开盘: 669.0
+最高: 680.0
+最低: 655.0
+收盘: 660.0</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 157 张 (占量 1.1%)
+          <t>法人净买超 157 张 (占量 1.3%)
 [2026-10-19 筹码] 主力机构呈净买入 (+157 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 670.0</t>
+          <t>NT$ 660.0</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>13,999 张</t>
+          <t>11,799 张</t>
         </is>
       </c>
     </row>
@@ -1513,10 +1513,10 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 4150.0
-最高: 4250.0
-最低: 4145.0
-收盘: 4205.0</t>
+          <t>开盘: 4260.0
+最高: 4305.0
+最低: 4120.0
+收盘: 4150.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 1,202 张 (占量 22.5%)
+          <t>法人净卖超 1,202 张 (占量 21.4%)
 [2026-10-19 筹码] 主力机构呈净卖出 (-1,202 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4205.0</t>
+          <t>NT$ 4150.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>5,350 张</t>
+          <t>5,612 张</t>
         </is>
       </c>
     </row>
@@ -1601,9 +1601,9 @@
       <c r="D14" s="7" t="inlineStr">
         <is>
           <t>开盘: 6475.0
-最高: 6590.0
-最低: 6330.0
-收盘: 6560.0</t>
+最高: 6720.0
+最低: 6475.0
+收盘: 6650.0</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 15 张 (占量 0.8%)
+          <t>法人净买超 15 张 (占量 1.7%)
 [2026-10-19 筹码] 主力机构呈净买入 (+15 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6560.0</t>
+          <t>NT$ 6650.0</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>1,857 张</t>
+          <t>876 张</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-19 21:46:09 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-20 15:06:07 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
+          <t>NT$ 2400.0</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2415.0</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
           <t>NT$ 2395.0</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2420.0</t>
-        </is>
-      </c>
-      <c r="E4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2390.0</t>
-        </is>
-      </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2420.0</t>
+          <t>NT$ 2405.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9785.0</t>
+          <t>NT$ 9985.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 10040.0</t>
+          <t>NT$ 10330.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9690.0</t>
+          <t>NT$ 9970.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9920.0</t>
+          <t>NT$ 10100.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5010.0</t>
+          <t>NT$ 5050.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5165.0</t>
+          <t>NT$ 5200.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 4955.0</t>
+          <t>NT$ 4930.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5125.0</t>
+          <t>NT$ 4945.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3220.0</t>
+          <t>NT$ 3290.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3350.0</t>
+          <t>NT$ 3420.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3180.0</t>
+          <t>NT$ 3270.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3320.0</t>
+          <t>NT$ 3325.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1960,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 242.0</t>
+          <t>NT$ 238.0</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 242.5</t>
+          <t>NT$ 244.5</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 238.5</t>
+          <t>NT$ 237.0</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 239.5</t>
+          <t>NT$ 241.5</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1600.0</t>
+          <t>NT$ 1635.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1655.0</t>
+          <t>NT$ 1645.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1590.0</t>
+          <t>NT$ 1595.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1640.0</t>
+          <t>NT$ 1605.0</t>
         </is>
       </c>
       <c r="G9" s="29" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1925.0</t>
+          <t>NT$ 2000.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
@@ -2064,12 +2064,12 @@
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1910.0</t>
+          <t>NT$ 1950.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2005.0</t>
+          <t>NT$ 1970.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2101,22 +2101,22 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1985.0</t>
+          <t>NT$ 2000.0</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2045.0</t>
+          <t>NT$ 2075.0</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1945.0</t>
+          <t>NT$ 1990.0</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2005.0</t>
+          <t>NT$ 2000.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 640.0</t>
+          <t>NT$ 669.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 675.0</t>
+          <t>NT$ 680.0</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 639.0</t>
+          <t>NT$ 655.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 670.0</t>
+          <t>NT$ 660.0</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
+          <t>NT$ 4260.0</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 4305.0</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 4120.0</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
           <t>NT$ 4150.0</t>
-        </is>
-      </c>
-      <c r="D13" s="28" t="inlineStr">
-        <is>
-          <t>NT$ 4250.0</t>
-        </is>
-      </c>
-      <c r="E13" s="28" t="inlineStr">
-        <is>
-          <t>NT$ 4145.0</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>NT$ 4205.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2247,17 +2247,17 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6590.0</t>
+          <t>NT$ 6720.0</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6330.0</t>
+          <t>NT$ 6475.0</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6560.0</t>
+          <t>NT$ 6650.0</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Publish October 21 close report and source freshness
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-20 19:55:25 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-21 15:06:14 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2400.0
-最高: 2415.0
-最低: 2395.0
-收盘: 2405.0</t>
+          <t>开盘: 2425.0
+最高: 2435.0
+最低: 2400.0
+收盘: 2420.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 8,364 张 (占量 49.1%)
+          <t>法人净卖超 8,364 张 (占量 37.5%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-8,364 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2405.0</t>
+          <t>NT$ 2420.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>17,029 张</t>
+          <t>22,276 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 9985.0
-最高: 10330.0
-最低: 9970.0
-收盘: 10100.0</t>
+          <t>开盘: 10500.0
+最高: 10580.0
+最低: 9985.0
+收盘: 10080.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 37 张 (占量 6.9%)
+          <t>法人净卖超 37 张 (占量 6.2%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-37 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 10100.0</t>
+          <t>NT$ 10080.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>533 张</t>
+          <t>592 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5050.0
-最高: 5200.0
-最低: 4930.0
-收盘: 4945.0</t>
+          <t>开盘: 5135.0
+最高: 5205.0
+最低: 4965.0
+收盘: 4990.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 193 张 (占量 12.2%)
+          <t>法人净卖超 193 张 (占量 7.6%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-193 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4945.0</t>
+          <t>NT$ 4990.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>1,585 张</t>
+          <t>2,537 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3290.0
-最高: 3420.0
-最低: 3270.0
-收盘: 3325.0</t>
+          <t>开盘: 3400.0
+最高: 3450.0
+最低: 3195.0
+收盘: 3235.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 209 张 (占量 7.9%)
+          <t>法人净买超 209 张 (占量 5.5%)
 [2026-10-20 筹码] 主力机构呈净买入 (+209 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3325.0</t>
+          <t>NT$ 3235.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,637 张</t>
+          <t>3,802 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 238.0
-最高: 244.5
-最低: 237.0
-收盘: 241.5</t>
+          <t>开盘: 244.5
+最高: 250.0
+最低: 244.5
+收盘: 250.0</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 5,218 张 (占量 19.9%)
+          <t>法人净买超 5,218 张 (占量 9.8%)
 [2026-10-20 筹码] 主力机构呈净买入 (+5,218 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 241.5</t>
+          <t>NT$ 250.0</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>26,229 张</t>
+          <t>53,380 张</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1165,10 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1635.0
-最高: 1645.0
-最低: 1595.0
-收盘: 1605.0</t>
+          <t>开盘: 1625.0
+最高: 1660.0
+最低: 1600.0
+收盘: 1625.0</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 3,275 张 (占量 41.2%)
+          <t>法人净卖超 3,275 张 (占量 31.1%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-3,275 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1605.0</t>
+          <t>NT$ 1625.0</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>7,947 张</t>
+          <t>10,519 张</t>
         </is>
       </c>
     </row>
@@ -1252,10 +1252,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2000.0
-最高: 2055.0
-最低: 1950.0
-收盘: 1970.0</t>
+          <t>开盘: 2045.0
+最高: 2050.0
+最低: 1805.0
+收盘: 1815.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 256 张 (占量 6.8%)
+          <t>法人净买超 256 张 (占量 3.6%)
 [2026-10-20 筹码] 主力机构呈净买入 (+256 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1970.0</t>
+          <t>NT$ 1815.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>3,781 张</t>
+          <t>7,140 张</t>
         </is>
       </c>
     </row>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>开盘: 2000.0
-最高: 2075.0
+          <t>开盘: 2030.0
+最高: 2095.0
 最低: 1990.0
-收盘: 2000.0</t>
+收盘: 2010.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 290 张 (占量 16.8%)
+          <t>法人净卖超 290 张 (占量 11.2%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-290 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2010.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>1,731 张</t>
+          <t>2,589 张</t>
         </is>
       </c>
     </row>
@@ -1426,10 +1426,10 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 669.0
-最高: 680.0
-最低: 655.0
-收盘: 660.0</t>
+          <t>开盘: 684.0
+最高: 687.0
+最低: 668.0
+收盘: 684.0</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 2,005 张 (占量 17.0%)
+          <t>法人净卖超 2,005 张 (占量 19.2%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-2,005 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 660.0</t>
+          <t>NT$ 684.0</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>11,799 张</t>
+          <t>10,425 张</t>
         </is>
       </c>
     </row>
@@ -1513,10 +1513,10 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 4260.0
-最高: 4305.0
-最低: 4120.0
-收盘: 4150.0</t>
+          <t>开盘: 4215.0
+最高: 4295.0
+最低: 4095.0
+收盘: 4140.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 1,368 张 (占量 24.4%)
+          <t>法人净卖超 1,368 张 (占量 17.1%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-1,368 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4150.0</t>
+          <t>NT$ 4140.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>5,612 张</t>
+          <t>8,018 张</t>
         </is>
       </c>
     </row>
@@ -1600,10 +1600,10 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>开盘: 6475.0
-最高: 6720.0
-最低: 6475.0
-收盘: 6650.0</t>
+          <t>开盘: 6835.0
+最高: 6985.0
+最低: 6500.0
+收盘: 6535.0</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 16 张 (占量 1.8%)
+          <t>法人净卖超 16 张 (占量 1.3%)
 [2026-10-20 筹码] 主力机构呈净卖出 (-16 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6650.0</t>
+          <t>NT$ 6535.0</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>876 张</t>
+          <t>1,271 张</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-20 19:55:25 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-21 15:06:14 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
+          <t>NT$ 2425.0</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 2435.0</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
           <t>NT$ 2400.0</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2415.0</t>
-        </is>
-      </c>
-      <c r="E4" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 2395.0</t>
-        </is>
-      </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2405.0</t>
+          <t>NT$ 2420.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
+          <t>NT$ 10500.0</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>NT$ 10580.0</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
           <t>NT$ 9985.0</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
-        <is>
-          <t>NT$ 10330.0</t>
-        </is>
-      </c>
-      <c r="E5" s="28" t="inlineStr">
-        <is>
-          <t>NT$ 9970.0</t>
-        </is>
-      </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 10100.0</t>
+          <t>NT$ 10080.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5050.0</t>
+          <t>NT$ 5135.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5200.0</t>
+          <t>NT$ 5205.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 4930.0</t>
+          <t>NT$ 4965.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4945.0</t>
+          <t>NT$ 4990.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3290.0</t>
+          <t>NT$ 3400.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3420.0</t>
+          <t>NT$ 3450.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3270.0</t>
+          <t>NT$ 3195.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3325.0</t>
+          <t>NT$ 3235.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1960,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 238.0</t>
+          <t>NT$ 244.5</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
+          <t>NT$ 250.0</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
           <t>NT$ 244.5</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 237.0</t>
-        </is>
-      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 241.5</t>
+          <t>NT$ 250.0</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1635.0</t>
+          <t>NT$ 1625.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1645.0</t>
+          <t>NT$ 1660.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1595.0</t>
+          <t>NT$ 1600.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1605.0</t>
+          <t>NT$ 1625.0</t>
         </is>
       </c>
       <c r="G9" s="29" t="inlineStr">
@@ -2054,22 +2054,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2045.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2055.0</t>
+          <t>NT$ 2050.0</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1950.0</t>
+          <t>NT$ 1805.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1970.0</t>
+          <t>NT$ 1815.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2101,12 +2101,12 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2030.0</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2075.0</t>
+          <t>NT$ 2095.0</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 2000.0</t>
+          <t>NT$ 2010.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 669.0</t>
+          <t>NT$ 684.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 680.0</t>
+          <t>NT$ 687.0</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 655.0</t>
+          <t>NT$ 668.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 660.0</t>
+          <t>NT$ 684.0</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4260.0</t>
+          <t>NT$ 4215.0</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4305.0</t>
+          <t>NT$ 4295.0</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4120.0</t>
+          <t>NT$ 4095.0</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4150.0</t>
+          <t>NT$ 4140.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2242,22 +2242,22 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6475.0</t>
+          <t>NT$ 6835.0</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6720.0</t>
+          <t>NT$ 6985.0</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6475.0</t>
+          <t>NT$ 6500.0</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6650.0</t>
+          <t>NT$ 6535.0</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Update daily stock report and source data for 2026-10-23
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-22 20:13:08 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-23 14:57:17 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-22 20:13:08 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-23 14:57:17 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: refresh October 24 disclosures and news with source gaps
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
auto: publish October 26 close report and source checks
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-23 19:54:13 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-26 15:03:33 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-23 19:54:13 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-26 15:03:33 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: publish October 27 close report and source gaps
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-26 21:25:08 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-27 15:04:06 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2435.0
-最高: 2435.0
-最低: 2385.0
-收盘: 2385.0</t>
+          <t>开盘: 2380.0
+最高: 2405.0
+最低: 2380.0
+收盘: 2400.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2385.0</t>
+          <t>NT$ 2400.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>22,750 张</t>
+          <t>33,882 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 10100.0
-最高: 10255.0
-最低: 9755.0
-收盘: 9755.0</t>
+          <t>开盘: 9830.0
+最高: 9890.0
+最低: 9475.0
+收盘: 9810.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9755.0</t>
+          <t>NT$ 9810.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>410 张</t>
+          <t>557 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5335.0
-最高: 5485.0
-最低: 5060.0
-收盘: 5070.0</t>
+          <t>开盘: 5200.0
+最高: 5200.0
+最低: 4685.0
+收盘: 4750.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5070.0</t>
+          <t>NT$ 4750.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>4,350 张</t>
+          <t>4,438 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3285.0
-最高: 3395.0
-最低: 3145.0
-收盘: 3145.0</t>
+          <t>开盘: 3300.0
+最高: 3320.0
+最低: 3050.0
+收盘: 3130.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3145.0</t>
+          <t>NT$ 3130.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,382 张</t>
+          <t>2,691 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 249.5
-最高: 250.5
-最低: 244.5
-收盘: 245.0</t>
+          <t>开盘: 246.5
+最高: 248.5
+最低: 244.0
+收盘: 247.5</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 245.0</t>
+          <t>NT$ 247.5</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>25,973 张</t>
+          <t>52,096 张</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1165,10 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1640.0
-最高: 1650.0
-最低: 1560.0
-收盘: 1560.0</t>
+          <t>开盘: 1535.0
+最高: 1570.0
+最低: 1490.0
+收盘: 1510.0</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1560.0</t>
+          <t>NT$ 1510.0</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>8,266 张</t>
+          <t>16,641 张</t>
         </is>
       </c>
     </row>
@@ -1252,10 +1252,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 1835.0
-最高: 1880.0
-最低: 1770.0
-收盘: 1775.0</t>
+          <t>开盘: 1760.0
+最高: 1805.0
+最低: 1740.0
+收盘: 1760.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1775.0</t>
+          <t>NT$ 1760.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>3,196 张</t>
+          <t>4,243 张</t>
         </is>
       </c>
     </row>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>开盘: 2090.0
-最高: 2110.0
-最低: 1975.0
-收盘: 1980.0</t>
+          <t>开盘: 1910.0
+最高: 1980.0
+最低: 1905.0
+收盘: 1955.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1980.0</t>
+          <t>NT$ 1955.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>2,170 张</t>
+          <t>3,549 张</t>
         </is>
       </c>
     </row>
@@ -1426,10 +1426,10 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 690.0
-最高: 699.0
-最低: 652.0
-收盘: 654.0</t>
+          <t>开盘: 654.0
+最高: 668.0
+最低: 642.0
+收盘: 651.0</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 654.0</t>
+          <t>NT$ 651.0</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>17,102 张</t>
+          <t>25,169 张</t>
         </is>
       </c>
     </row>
@@ -1513,10 +1513,10 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 4230.0
-最高: 4230.0
-最低: 4005.0
-收盘: 4010.0</t>
+          <t>开盘: 4035.0
+最高: 4075.0
+最低: 3910.0
+收盘: 3960.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4010.0</t>
+          <t>NT$ 3960.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>5,885 张</t>
+          <t>11,978 张</t>
         </is>
       </c>
     </row>
@@ -1600,10 +1600,10 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>开盘: 6555.0
-最高: 6675.0
-最低: 5995.0
-收盘: 6070.0</t>
+          <t>开盘: 6080.0
+最高: 6095.0
+最低: 5710.0
+收盘: 5860.0</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6070.0</t>
+          <t>NT$ 5860.0</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>1,645 张</t>
+          <t>2,354 张</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-26 21:25:08 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-27 15:04:06 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2435.0</t>
+          <t>NT$ 2380.0</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2435.0</t>
+          <t>NT$ 2405.0</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2385.0</t>
+          <t>NT$ 2380.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2385.0</t>
+          <t>NT$ 2400.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 10100.0</t>
+          <t>NT$ 9830.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 10255.0</t>
+          <t>NT$ 9890.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9755.0</t>
+          <t>NT$ 9475.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9755.0</t>
+          <t>NT$ 9810.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5335.0</t>
+          <t>NT$ 5200.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5485.0</t>
+          <t>NT$ 5200.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5060.0</t>
+          <t>NT$ 4685.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5070.0</t>
+          <t>NT$ 4750.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3285.0</t>
+          <t>NT$ 3300.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3395.0</t>
+          <t>NT$ 3320.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3145.0</t>
+          <t>NT$ 3050.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3145.0</t>
+          <t>NT$ 3130.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1960,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 249.5</t>
+          <t>NT$ 246.5</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 250.5</t>
+          <t>NT$ 248.5</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>NT$ 244.5</t>
+          <t>NT$ 244.0</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 245.0</t>
+          <t>NT$ 247.5</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1640.0</t>
+          <t>NT$ 1535.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1650.0</t>
+          <t>NT$ 1570.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1560.0</t>
+          <t>NT$ 1490.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1560.0</t>
+          <t>NT$ 1510.0</t>
         </is>
       </c>
       <c r="G9" s="29" t="inlineStr">
@@ -2054,22 +2054,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1835.0</t>
+          <t>NT$ 1760.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1880.0</t>
+          <t>NT$ 1805.0</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1770.0</t>
+          <t>NT$ 1740.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1775.0</t>
+          <t>NT$ 1760.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2101,22 +2101,22 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2090.0</t>
+          <t>NT$ 1910.0</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 2110.0</t>
+          <t>NT$ 1980.0</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1975.0</t>
+          <t>NT$ 1905.0</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1980.0</t>
+          <t>NT$ 1955.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 690.0</t>
+          <t>NT$ 654.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 699.0</t>
+          <t>NT$ 668.0</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 652.0</t>
+          <t>NT$ 642.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 654.0</t>
+          <t>NT$ 651.0</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4230.0</t>
+          <t>NT$ 4035.0</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4230.0</t>
+          <t>NT$ 4075.0</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4005.0</t>
+          <t>NT$ 3910.0</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 4010.0</t>
+          <t>NT$ 3960.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2242,22 +2242,22 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6555.0</t>
+          <t>NT$ 6080.0</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6675.0</t>
+          <t>NT$ 6095.0</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5995.0</t>
+          <t>NT$ 5710.0</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 6070.0</t>
+          <t>NT$ 5860.0</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Publish October 28 close report with verified source dates
</commit_message>
<xml_diff>
--- a/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
+++ b/台股 5 大 AI 核心卡位龙头深度投资与买卖点筹码量化分析表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心卡位龙头全景深度分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="买卖决策速查面板" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -631,7 +631,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>定盘时间: 2026-10-27 20:31:24 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
+          <t>定盘时间: 2026-10-28 14:57:18 | 数据源: Shioaji Snapshot (primary) + TWSE MIS cross-check | 包含三大法人买卖超、财报发布日及主力资金分析</t>
         </is>
       </c>
     </row>
@@ -730,10 +730,10 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>开盘: 2380.0
-最高: 2405.0
-最低: 2380.0
-收盘: 2400.0</t>
+          <t>开盘: 2420.0
+最高: 2430.0
+最低: 2410.0
+收盘: 2425.0</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 2,709 张 (占量 8.0%)
+          <t>法人净买超 2,709 张 (占量 13.6%)
 [2026-10-27 筹码] 主力机构呈净买入 (+2,709 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -769,7 +769,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2400.0</t>
+          <t>NT$ 2425.0</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>33,882 张</t>
+          <t>19,852 张</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>开盘: 9830.0
-最高: 9890.0
-最低: 9475.0
-收盘: 9810.0</t>
+          <t>开盘: 10225.0
+最高: 10290.0
+最低: 10015.0
+收盘: 10150.0</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="H5" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 108 张 (占量 19.4%)
+          <t>法人净买超 108 张 (占量 35.4%)
 [2026-10-27 筹码] 主力机构呈净买入 (+108 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -856,7 +856,7 @@
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9810.0</t>
+          <t>NT$ 10150.0</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="O5" s="16" t="inlineStr">
         <is>
-          <t>557 张</t>
+          <t>305 张</t>
         </is>
       </c>
     </row>
@@ -904,10 +904,10 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>开盘: 5200.0
-最高: 5200.0
-最低: 4685.0
-收盘: 4750.0</t>
+          <t>开盘: 4975.0
+最高: 5065.0
+最低: 4830.0
+收盘: 5025.0</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 760 张 (占量 17.1%)
+          <t>法人净卖超 760 张 (占量 24.3%)
 [2026-10-27 筹码] 主力机构呈净卖出 (-760 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -943,7 +943,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4750.0</t>
+          <t>NT$ 5025.0</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>4,438 张</t>
+          <t>3,130 张</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,10 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>开盘: 3300.0
-最高: 3320.0
-最低: 3050.0
-收盘: 3130.0</t>
+          <t>开盘: 3230.0
+最高: 3330.0
+最低: 3185.0
+收盘: 3215.0</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H7" s="15" t="inlineStr">
         <is>
-          <t>法人净买超 126 张 (占量 4.7%)
+          <t>法人净买超 126 张 (占量 6.2%)
 [2026-10-27 筹码] 主力机构呈净买入 (+126 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3130.0</t>
+          <t>NT$ 3215.0</t>
         </is>
       </c>
       <c r="K7" s="18" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>2,691 张</t>
+          <t>2,024 张</t>
         </is>
       </c>
     </row>
@@ -1078,10 +1078,10 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>开盘: 246.5
-最高: 248.5
-最低: 244.0
-收盘: 247.5</t>
+          <t>开盘: 248.0
+最高: 252.0
+最低: 246.5
+收盘: 251.5</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 7,123 张 (占量 13.7%)
+          <t>法人净买超 7,123 张 (占量 17.2%)
 [2026-10-27 筹码] 主力机构呈净买入 (+7,123 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 247.5</t>
+          <t>NT$ 251.5</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
-          <t>52,096 张</t>
+          <t>41,355 张</t>
         </is>
       </c>
     </row>
@@ -1165,10 +1165,10 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1535.0
-最高: 1570.0
-最低: 1490.0
-收盘: 1510.0</t>
+          <t>开盘: 1565.0
+最高: 1575.0
+最低: 1515.0
+收盘: 1550.0</t>
         </is>
       </c>
       <c r="E9" s="15" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 2,662 张 (占量 16.0%)
+          <t>法人净卖超 2,662 张 (占量 38.4%)
 [2026-10-27 筹码] 主力机构呈净卖出 (-2,662 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1510.0</t>
+          <t>NT$ 1550.0</t>
         </is>
       </c>
       <c r="K9" s="18" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="O9" s="16" t="inlineStr">
         <is>
-          <t>16,641 张</t>
+          <t>6,925 张</t>
         </is>
       </c>
     </row>
@@ -1252,10 +1252,10 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>开盘: 1760.0
-最高: 1805.0
-最低: 1740.0
-收盘: 1760.0</t>
+          <t>开盘: 1820.0
+最高: 1830.0
+最低: 1780.0
+收盘: 1815.0</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 552 张 (占量 13.0%)
+          <t>法人净买超 552 张 (占量 19.1%)
 [2026-10-27 筹码] 主力机构呈净买入 (+552 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1760.0</t>
+          <t>NT$ 1815.0</t>
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>4,243 张</t>
+          <t>2,889 张</t>
         </is>
       </c>
     </row>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>开盘: 1910.0
-最高: 1980.0
-最低: 1905.0
-收盘: 1955.0</t>
+          <t>开盘: 1995.0
+最高: 2050.0
+最低: 1995.0
+收盘: 2035.0</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 42 张 (占量 1.2%)
+          <t>法人净卖超 42 张 (占量 1.0%)
 [2026-10-27 筹码] 主力机构呈净卖出 (-42 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1955.0</t>
+          <t>NT$ 2035.0</t>
         </is>
       </c>
       <c r="K11" s="18" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="O11" s="16" t="inlineStr">
         <is>
-          <t>3,549 张</t>
+          <t>4,050 张</t>
         </is>
       </c>
     </row>
@@ -1426,10 +1426,10 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>开盘: 654.0
-最高: 668.0
-最低: 642.0
-收盘: 651.0</t>
+          <t>开盘: 672.0
+最高: 698.0
+最低: 672.0
+收盘: 695.0</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>法人净卖超 850 张 (占量 3.4%)
+          <t>法人净卖超 850 张 (占量 4.5%)
 [2026-10-27 筹码] 主力机构呈净卖出 (-850 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 651.0</t>
+          <t>NT$ 695.0</t>
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>25,169 张</t>
+          <t>18,912 张</t>
         </is>
       </c>
     </row>
@@ -1513,10 +1513,10 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>开盘: 4035.0
-最高: 4075.0
-最低: 3910.0
-收盘: 3960.0</t>
+          <t>开盘: 4040.0
+最高: 4245.0
+最低: 4040.0
+收盘: 4235.0</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>法人净卖超 1,492 张 (占量 12.5%)
+          <t>法人净卖超 1,492 张 (占量 21.5%)
 [2026-10-27 筹码] 主力机构呈净卖出 (-1,492 张)，散户承接，筹码短期发散。</t>
         </is>
       </c>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3960.0</t>
+          <t>NT$ 4235.0</t>
         </is>
       </c>
       <c r="K13" s="18" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O13" s="16" t="inlineStr">
         <is>
-          <t>11,978 张</t>
+          <t>6,953 张</t>
         </is>
       </c>
     </row>
@@ -1600,10 +1600,10 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>开盘: 6080.0
-最高: 6095.0
-最低: 5710.0
-收盘: 5860.0</t>
+          <t>开盘: 6200.0
+最高: 6445.0
+最低: 6055.0
+收盘: 6375.0</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>法人净买超 857 张 (占量 36.4%)
+          <t>法人净买超 857 张 (占量 40.2%)
 [2026-10-27 筹码] 主力机构呈净买入 (+857 张)，筹码向法人端汇聚沉淀。</t>
         </is>
       </c>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5860.0</t>
+          <t>NT$ 6375.0</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>2,354 张</t>
+          <t>2,130 张</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-27 20:31:24 | 策略: 3-3-4 分批建仓</t>
+          <t>数据源: 永丰金 Shioaji 实时盘口 | 定盘时间: 2026-10-28 14:57:18 | 策略: 3-3-4 分批建仓</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2380.0</t>
+          <t>NT$ 2420.0</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2405.0</t>
+          <t>NT$ 2430.0</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>NT$ 2380.0</t>
+          <t>NT$ 2410.0</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>NT$ 2400.0</t>
+          <t>NT$ 2425.0</t>
         </is>
       </c>
       <c r="G4" s="25" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9830.0</t>
+          <t>NT$ 10225.0</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9890.0</t>
+          <t>NT$ 10290.0</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
         <is>
-          <t>NT$ 9475.0</t>
+          <t>NT$ 10015.0</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>NT$ 9810.0</t>
+          <t>NT$ 10150.0</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5200.0</t>
+          <t>NT$ 4975.0</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5200.0</t>
+          <t>NT$ 5065.0</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>NT$ 4685.0</t>
+          <t>NT$ 4830.0</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>NT$ 4750.0</t>
+          <t>NT$ 5025.0</t>
         </is>
       </c>
       <c r="G6" s="25" t="inlineStr">
@@ -1913,22 +1913,22 @@
       </c>
       <c r="C7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3300.0</t>
+          <t>NT$ 3230.0</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3320.0</t>
+          <t>NT$ 3330.0</t>
         </is>
       </c>
       <c r="E7" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3050.0</t>
+          <t>NT$ 3185.0</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3130.0</t>
+          <t>NT$ 3215.0</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
@@ -1960,22 +1960,22 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
+          <t>NT$ 248.0</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>NT$ 252.0</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
           <t>NT$ 246.5</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 248.5</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>NT$ 244.0</t>
-        </is>
-      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>NT$ 247.5</t>
+          <t>NT$ 251.5</t>
         </is>
       </c>
       <c r="G8" s="25" t="inlineStr">
@@ -2007,22 +2007,22 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1535.0</t>
+          <t>NT$ 1565.0</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1570.0</t>
+          <t>NT$ 1575.0</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1490.0</t>
+          <t>NT$ 1515.0</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1510.0</t>
+          <t>NT$ 1550.0</t>
         </is>
       </c>
       <c r="G9" s="29" t="inlineStr">
@@ -2054,22 +2054,22 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1760.0</t>
+          <t>NT$ 1820.0</t>
         </is>
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1805.0</t>
+          <t>NT$ 1830.0</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>NT$ 1740.0</t>
+          <t>NT$ 1780.0</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>NT$ 1760.0</t>
+          <t>NT$ 1815.0</t>
         </is>
       </c>
       <c r="G10" s="25" t="inlineStr">
@@ -2101,22 +2101,22 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1910.0</t>
+          <t>NT$ 1995.0</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1980.0</t>
+          <t>NT$ 2050.0</t>
         </is>
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
-          <t>NT$ 1905.0</t>
+          <t>NT$ 1995.0</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>NT$ 1955.0</t>
+          <t>NT$ 2035.0</t>
         </is>
       </c>
       <c r="G11" s="29" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 654.0</t>
+          <t>NT$ 672.0</t>
         </is>
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 668.0</t>
+          <t>NT$ 698.0</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>NT$ 642.0</t>
+          <t>NT$ 672.0</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>NT$ 651.0</t>
+          <t>NT$ 695.0</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2195,22 +2195,22 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4035.0</t>
+          <t>NT$ 4040.0</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 4075.0</t>
+          <t>NT$ 4245.0</t>
         </is>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
-          <t>NT$ 3910.0</t>
+          <t>NT$ 4040.0</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>NT$ 3960.0</t>
+          <t>NT$ 4235.0</t>
         </is>
       </c>
       <c r="G13" s="29" t="inlineStr">
@@ -2242,22 +2242,22 @@
       </c>
       <c r="C14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6080.0</t>
+          <t>NT$ 6200.0</t>
         </is>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 6095.0</t>
+          <t>NT$ 6445.0</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>NT$ 5710.0</t>
+          <t>NT$ 6055.0</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>NT$ 5860.0</t>
+          <t>NT$ 6375.0</t>
         </is>
       </c>
       <c r="G14" s="25" t="inlineStr">

</xml_diff>